<commit_message>
Shuffle Whats-This answers to balanced distribution
</commit_message>
<xml_diff>
--- a/whats-this-quiz/Kahoot-Whats-This.xlsx
+++ b/whats-this-quiz/Kahoot-Whats-This.xlsx
@@ -712,17 +712,17 @@
       </c>
       <c r="C9" s="22" t="inlineStr">
         <is>
+          <t>Duck Show</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>Lion Show</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
           <t>What's This?</t>
-        </is>
-      </c>
-      <c r="D9" s="22" t="inlineStr">
-        <is>
-          <t>Duck Show</t>
-        </is>
-      </c>
-      <c r="E9" s="22" t="inlineStr">
-        <is>
-          <t>Lion Show</t>
         </is>
       </c>
       <c r="F9" s="22" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="H9" s="23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I9" s="1" t="n"/>
@@ -751,12 +751,12 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
           <t>Judy</t>
-        </is>
-      </c>
-      <c r="D10" s="25" t="inlineStr">
-        <is>
-          <t>David</t>
         </is>
       </c>
       <c r="E10" s="25" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H10" s="26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" s="1" t="n"/>
@@ -790,22 +790,22 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
+          <t>A duck</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>A monkey</t>
+        </is>
+      </c>
+      <c r="E11" s="25" t="inlineStr">
+        <is>
+          <t>A tiger</t>
+        </is>
+      </c>
+      <c r="F11" s="25" t="inlineStr">
+        <is>
           <t>A goose</t>
-        </is>
-      </c>
-      <c r="D11" s="25" t="inlineStr">
-        <is>
-          <t>A duck</t>
-        </is>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>A monkey</t>
-        </is>
-      </c>
-      <c r="F11" s="25" t="inlineStr">
-        <is>
-          <t>A tiger</t>
         </is>
       </c>
       <c r="G11" s="25" t="n">
@@ -813,7 +813,7 @@
       </c>
       <c r="H11" s="26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I11" s="1" t="n"/>
@@ -868,12 +868,12 @@
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
+          <t>Lions</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
           <t>Tigers</t>
-        </is>
-      </c>
-      <c r="D13" s="25" t="inlineStr">
-        <is>
-          <t>Lions</t>
         </is>
       </c>
       <c r="E13" s="25" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="H13" s="26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" s="1" t="n"/>
@@ -907,22 +907,22 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
+          <t>big duck</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>small lion</t>
+        </is>
+      </c>
+      <c r="E14" s="25" t="inlineStr">
+        <is>
+          <t>tired monkey</t>
+        </is>
+      </c>
+      <c r="F14" s="25" t="inlineStr">
+        <is>
           <t>smart cookie</t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="inlineStr">
-        <is>
-          <t>big duck</t>
-        </is>
-      </c>
-      <c r="E14" s="25" t="inlineStr">
-        <is>
-          <t>small lion</t>
-        </is>
-      </c>
-      <c r="F14" s="25" t="inlineStr">
-        <is>
-          <t>tired monkey</t>
         </is>
       </c>
       <c r="G14" s="25" t="n">
@@ -930,7 +930,7 @@
       </c>
       <c r="H14" s="26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I14" s="1" t="n"/>
@@ -946,17 +946,17 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
+          <t>Yes, that's it</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="inlineStr">
+        <is>
+          <t>Yes, ten points</t>
+        </is>
+      </c>
+      <c r="E15" s="25" t="inlineStr">
+        <is>
           <t>No, sorry</t>
-        </is>
-      </c>
-      <c r="D15" s="25" t="inlineStr">
-        <is>
-          <t>Yes, that's it</t>
-        </is>
-      </c>
-      <c r="E15" s="25" t="inlineStr">
-        <is>
-          <t>Yes, ten points</t>
         </is>
       </c>
       <c r="F15" s="25" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="H15" s="26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I15" s="1" t="n"/>
@@ -985,12 +985,12 @@
       </c>
       <c r="C16" s="25" t="inlineStr">
         <is>
+          <t>A monkey</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="inlineStr">
+        <is>
           <t>Bigfoot</t>
-        </is>
-      </c>
-      <c r="D16" s="25" t="inlineStr">
-        <is>
-          <t>A monkey</t>
         </is>
       </c>
       <c r="E16" s="25" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H16" s="26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" s="1" t="n"/>
@@ -1024,22 +1024,22 @@
       </c>
       <c r="C17" s="25" t="inlineStr">
         <is>
+          <t>gooses</t>
+        </is>
+      </c>
+      <c r="D17" s="25" t="inlineStr">
+        <is>
+          <t>goose</t>
+        </is>
+      </c>
+      <c r="E17" s="25" t="inlineStr">
+        <is>
+          <t>geeses</t>
+        </is>
+      </c>
+      <c r="F17" s="25" t="inlineStr">
+        <is>
           <t>geese</t>
-        </is>
-      </c>
-      <c r="D17" s="25" t="inlineStr">
-        <is>
-          <t>gooses</t>
-        </is>
-      </c>
-      <c r="E17" s="25" t="inlineStr">
-        <is>
-          <t>goose</t>
-        </is>
-      </c>
-      <c r="F17" s="25" t="inlineStr">
-        <is>
-          <t>geeses</t>
         </is>
       </c>
       <c r="G17" s="25" t="n">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="H17" s="26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I17" s="1" t="n"/>

</xml_diff>